<commit_message>
docs: model charts change
</commit_message>
<xml_diff>
--- a/src/logging_record/ablation.xlsx
+++ b/src/logging_record/ablation.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10312"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10420"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/lbp/Desktop/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/huangdenan/github/personal_github/Causal3D-Net/src/logging_record/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{6704CD45-B6DB-A84A-9BC4-BEF71983DFF0}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="36" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D254B310-4306-7648-AA98-6D33DFD21496}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="280" yWindow="460" windowWidth="28240" windowHeight="16400" xr2:uid="{0674E527-E1AB-E348-9FF3-CA6262F7D631}"/>
+    <workbookView xWindow="160" yWindow="660" windowWidth="50880" windowHeight="26400" xr2:uid="{0674E527-E1AB-E348-9FF3-CA6262F7D631}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -24,9 +24,142 @@
 </workbook>
 </file>
 
+<file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="97" uniqueCount="31">
+  <si>
+    <t>individual_branch</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>center_branch</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>orthogonal</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>Accuracy</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>AUC</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>Sensitivity</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>Specificity</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>Precision</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>F1</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>date</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>2025-06-29_14-02-40</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>2025-06-26_11-57-43</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>2025-06-30_13-20-41</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>2025-07-04_11-36-01</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>2025-07-04_22-44-30</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>2025-07-05_09-57-18</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>dataset</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>2025-06-30_01-48-53</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>name</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>baseline</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>indi</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>cent</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>indi+cent</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>Note</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>CV set</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>test I</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>test II</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>test III</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>indi+ot</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>cent+ot</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>indi+cent+ot</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+</sst>
+</file>
+
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="2">
+  <numFmts count="2">
+    <numFmt numFmtId="176" formatCode="0.000"/>
+    <numFmt numFmtId="177" formatCode="0.0000"/>
+  </numFmts>
+  <fonts count="3">
     <font>
       <sz val="12"/>
       <color theme="1"/>
@@ -42,21 +175,68 @@
       <charset val="134"/>
       <scheme val="minor"/>
     </font>
+    <font>
+      <sz val="12"/>
+      <color rgb="FF000000"/>
+      <name val="等线"/>
+      <family val="4"/>
+      <charset val="134"/>
+      <scheme val="minor"/>
+    </font>
   </fonts>
-  <fills count="2">
+  <fills count="6">
     <fill>
       <patternFill patternType="none"/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="9" tint="0.59999389629810485"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="8" tint="0.59999389629810485"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="7" tint="0.59999389629810485"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="6" tint="0.59999389629810485"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
   </fills>
-  <borders count="1">
+  <borders count="2">
     <border>
       <left/>
       <right/>
       <top/>
       <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
       <diagonal/>
     </border>
   </borders>
@@ -65,8 +245,41 @@
       <alignment vertical="center"/>
     </xf>
   </cellStyleXfs>
-  <cellXfs count="1">
+  <cellXfs count="12">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="1" xfId="0" applyFill="1" applyBorder="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="1" xfId="0" applyFill="1" applyBorder="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="1" xfId="0" applyFill="1" applyBorder="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="177" fontId="0" fillId="4" borderId="1" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="5" borderId="1" xfId="0" applyFill="1" applyBorder="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="177" fontId="0" fillId="5" borderId="1" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="176" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="177" fontId="0" fillId="2" borderId="1" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="177" fontId="0" fillId="3" borderId="1" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="177" fontId="2" fillId="3" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1">
       <alignment vertical="center"/>
     </xf>
   </cellXfs>
@@ -87,9 +300,9 @@
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
-<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office 主题​​">
+<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office 2013 - 2022 主题">
   <a:themeElements>
-    <a:clrScheme name="Office">
+    <a:clrScheme name="Office 2013 - 2022">
       <a:dk1>
         <a:sysClr val="windowText" lastClr="000000"/>
       </a:dk1>
@@ -127,7 +340,7 @@
         <a:srgbClr val="954F72"/>
       </a:folHlink>
     </a:clrScheme>
-    <a:fontScheme name="Office">
+    <a:fontScheme name="Office 2013 - 2022">
       <a:majorFont>
         <a:latin typeface="Calibri Light" panose="020F0302020204030204"/>
         <a:ea typeface=""/>
@@ -233,7 +446,7 @@
         <a:font script="Tfng" typeface="Ebrima"/>
       </a:minorFont>
     </a:fontScheme>
-    <a:fmtScheme name="Office">
+    <a:fmtScheme name="Office 2013 - 2022">
       <a:fillStyleLst>
         <a:solidFill>
           <a:schemeClr val="phClr"/>
@@ -375,7 +588,7 @@
   <a:extraClrSchemeLst/>
   <a:extLst>
     <a:ext uri="{05A4C25C-085E-4340-85A3-A5531E510DB2}">
-      <thm15:themeFamily xmlns:thm15="http://schemas.microsoft.com/office/thememl/2012/main" name="Office Theme" id="{62F939B6-93AF-4DB8-9C6B-D6C7DFDC589F}" vid="{4A3C46E8-61CC-4603-A589-7422A47A8E4A}"/>
+      <thm15:themeFamily xmlns:thm15="http://schemas.microsoft.com/office/thememl/2012/main" name="Office 2013 - 2022 Theme" id="{62F939B6-93AF-4DB8-9C6B-D6C7DFDC589F}" vid="{4A3C46E8-61CC-4603-A589-7422A47A8E4A}"/>
     </a:ext>
   </a:extLst>
 </a:theme>
@@ -383,10 +596,1204 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{F25302E3-D780-C043-8AFB-452B651797D6}">
-  <dimension ref="A1"/>
+  <dimension ref="A1:N45"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16"/>
-  <sheetData/>
+  <cols>
+    <col min="1" max="1" width="28.83203125" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="21.83203125" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="18" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="14.33203125" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="11.83203125" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="8.33203125" bestFit="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:14">
+      <c r="A1" s="1" t="s">
+        <v>18</v>
+      </c>
+      <c r="B1" s="1" t="s">
+        <v>9</v>
+      </c>
+      <c r="C1" s="1" t="s">
+        <v>0</v>
+      </c>
+      <c r="D1" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="E1" s="1" t="s">
+        <v>2</v>
+      </c>
+      <c r="F1" s="1" t="s">
+        <v>16</v>
+      </c>
+      <c r="G1" s="1" t="s">
+        <v>3</v>
+      </c>
+      <c r="H1" s="1" t="s">
+        <v>4</v>
+      </c>
+      <c r="I1" s="1" t="s">
+        <v>5</v>
+      </c>
+      <c r="J1" s="1" t="s">
+        <v>6</v>
+      </c>
+      <c r="K1" s="1" t="s">
+        <v>7</v>
+      </c>
+      <c r="L1" s="1" t="s">
+        <v>8</v>
+      </c>
+      <c r="M1" s="1" t="s">
+        <v>23</v>
+      </c>
+    </row>
+    <row r="2" spans="1:14">
+      <c r="A2" s="2" t="s">
+        <v>19</v>
+      </c>
+      <c r="B2" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="C2" s="2">
+        <v>0</v>
+      </c>
+      <c r="D2" s="2">
+        <v>0</v>
+      </c>
+      <c r="E2" s="2">
+        <v>1</v>
+      </c>
+      <c r="F2" s="2" t="s">
+        <v>24</v>
+      </c>
+      <c r="G2" s="9">
+        <v>0.91300000000000003</v>
+      </c>
+      <c r="H2" s="9">
+        <v>0.97009999999999996</v>
+      </c>
+      <c r="I2" s="9">
+        <v>0.89170000000000005</v>
+      </c>
+      <c r="J2" s="9">
+        <v>0.9274</v>
+      </c>
+      <c r="K2" s="9">
+        <v>0.89170000000000005</v>
+      </c>
+      <c r="L2" s="9">
+        <v>0.89170000000000005</v>
+      </c>
+      <c r="M2" s="1">
+        <v>24</v>
+      </c>
+      <c r="N2" s="8"/>
+    </row>
+    <row r="3" spans="1:14">
+      <c r="A3" s="2" t="s">
+        <v>20</v>
+      </c>
+      <c r="B3" s="2" t="s">
+        <v>13</v>
+      </c>
+      <c r="C3" s="2">
+        <v>1</v>
+      </c>
+      <c r="D3" s="2">
+        <v>0</v>
+      </c>
+      <c r="E3" s="2">
+        <v>0</v>
+      </c>
+      <c r="F3" s="2" t="s">
+        <v>24</v>
+      </c>
+      <c r="G3" s="9">
+        <v>0.91010000000000002</v>
+      </c>
+      <c r="H3" s="9">
+        <v>0.96660000000000001</v>
+      </c>
+      <c r="I3" s="9">
+        <v>0.88219999999999998</v>
+      </c>
+      <c r="J3" s="9">
+        <v>0.92879999999999996</v>
+      </c>
+      <c r="K3" s="9">
+        <v>0.89259999999999995</v>
+      </c>
+      <c r="L3" s="9">
+        <v>0.88729999999999998</v>
+      </c>
+      <c r="M3" s="1">
+        <v>37</v>
+      </c>
+    </row>
+    <row r="4" spans="1:14">
+      <c r="A4" s="2" t="s">
+        <v>28</v>
+      </c>
+      <c r="B4" s="2" t="s">
+        <v>10</v>
+      </c>
+      <c r="C4" s="2">
+        <v>1</v>
+      </c>
+      <c r="D4" s="2">
+        <v>0</v>
+      </c>
+      <c r="E4" s="2">
+        <v>1</v>
+      </c>
+      <c r="F4" s="2" t="s">
+        <v>24</v>
+      </c>
+      <c r="G4" s="9">
+        <v>0.87470000000000003</v>
+      </c>
+      <c r="H4" s="9">
+        <v>0.94599999999999995</v>
+      </c>
+      <c r="I4" s="9">
+        <v>0.86939999999999995</v>
+      </c>
+      <c r="J4" s="9">
+        <v>0.87819999999999998</v>
+      </c>
+      <c r="K4" s="9">
+        <v>0.82730000000000004</v>
+      </c>
+      <c r="L4" s="9">
+        <v>0.8478</v>
+      </c>
+      <c r="M4" s="1">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="5" spans="1:14">
+      <c r="A5" s="2" t="s">
+        <v>21</v>
+      </c>
+      <c r="B5" s="2" t="s">
+        <v>14</v>
+      </c>
+      <c r="C5" s="2">
+        <v>0</v>
+      </c>
+      <c r="D5" s="2">
+        <v>1</v>
+      </c>
+      <c r="E5" s="2">
+        <v>0</v>
+      </c>
+      <c r="F5" s="2" t="s">
+        <v>24</v>
+      </c>
+      <c r="G5" s="9">
+        <v>0.91520000000000001</v>
+      </c>
+      <c r="H5" s="9">
+        <v>0.96789999999999998</v>
+      </c>
+      <c r="I5" s="9">
+        <v>0.88319999999999999</v>
+      </c>
+      <c r="J5" s="9">
+        <v>0.93659999999999999</v>
+      </c>
+      <c r="K5" s="9">
+        <v>0.90339999999999998</v>
+      </c>
+      <c r="L5" s="9">
+        <v>0.89319999999999999</v>
+      </c>
+      <c r="M5" s="1">
+        <v>31</v>
+      </c>
+    </row>
+    <row r="6" spans="1:14">
+      <c r="A6" s="2" t="s">
+        <v>29</v>
+      </c>
+      <c r="B6" s="2" t="s">
+        <v>17</v>
+      </c>
+      <c r="C6" s="2">
+        <v>0</v>
+      </c>
+      <c r="D6" s="2">
+        <v>1</v>
+      </c>
+      <c r="E6" s="2">
+        <v>1</v>
+      </c>
+      <c r="F6" s="2" t="s">
+        <v>24</v>
+      </c>
+      <c r="G6" s="9">
+        <v>0.93089999999999995</v>
+      </c>
+      <c r="H6" s="9">
+        <v>0.97809999999999997</v>
+      </c>
+      <c r="I6" s="9">
+        <v>0.9002</v>
+      </c>
+      <c r="J6" s="9">
+        <v>0.9516</v>
+      </c>
+      <c r="K6" s="9">
+        <v>0.92579999999999996</v>
+      </c>
+      <c r="L6" s="9">
+        <v>0.91279999999999994</v>
+      </c>
+      <c r="M6" s="1">
+        <v>31</v>
+      </c>
+    </row>
+    <row r="7" spans="1:14">
+      <c r="A7" s="2" t="s">
+        <v>22</v>
+      </c>
+      <c r="B7" s="2" t="s">
+        <v>15</v>
+      </c>
+      <c r="C7" s="2">
+        <v>1</v>
+      </c>
+      <c r="D7" s="2">
+        <v>1</v>
+      </c>
+      <c r="E7" s="2">
+        <v>0</v>
+      </c>
+      <c r="F7" s="2" t="s">
+        <v>24</v>
+      </c>
+      <c r="G7" s="9">
+        <v>0.9365</v>
+      </c>
+      <c r="H7" s="9">
+        <v>0.98229999999999995</v>
+      </c>
+      <c r="I7" s="9">
+        <v>0.91190000000000004</v>
+      </c>
+      <c r="J7" s="9">
+        <v>0.95299999999999996</v>
+      </c>
+      <c r="K7" s="9">
+        <v>0.92859999999999998</v>
+      </c>
+      <c r="L7" s="9">
+        <v>0.92020000000000002</v>
+      </c>
+      <c r="M7" s="1"/>
+    </row>
+    <row r="8" spans="1:14">
+      <c r="A8" s="2" t="s">
+        <v>30</v>
+      </c>
+      <c r="B8" s="2" t="s">
+        <v>11</v>
+      </c>
+      <c r="C8" s="2">
+        <v>1</v>
+      </c>
+      <c r="D8" s="2">
+        <v>1</v>
+      </c>
+      <c r="E8" s="2">
+        <v>1</v>
+      </c>
+      <c r="F8" s="2" t="s">
+        <v>24</v>
+      </c>
+      <c r="G8" s="9">
+        <v>0.89132933260592795</v>
+      </c>
+      <c r="H8" s="9">
+        <v>0.94659456245865903</v>
+      </c>
+      <c r="I8" s="9">
+        <v>0.84799999999999998</v>
+      </c>
+      <c r="J8" s="9">
+        <v>0.92028875379939201</v>
+      </c>
+      <c r="K8" s="9">
+        <v>0.87980962438462496</v>
+      </c>
+      <c r="L8" s="9">
+        <v>0.86257597988225798</v>
+      </c>
+      <c r="M8" s="1"/>
+    </row>
+    <row r="9" spans="1:14">
+      <c r="A9" s="3" t="s">
+        <v>19</v>
+      </c>
+      <c r="B9" s="3" t="s">
+        <v>12</v>
+      </c>
+      <c r="C9" s="3">
+        <v>0</v>
+      </c>
+      <c r="D9" s="3">
+        <v>0</v>
+      </c>
+      <c r="E9" s="3">
+        <v>1</v>
+      </c>
+      <c r="F9" s="3" t="s">
+        <v>25</v>
+      </c>
+      <c r="G9" s="10">
+        <v>0.89090000000000003</v>
+      </c>
+      <c r="H9" s="10">
+        <v>0.94589999999999996</v>
+      </c>
+      <c r="I9" s="10">
+        <v>0.97850000000000004</v>
+      </c>
+      <c r="J9" s="10">
+        <v>0.77780000000000005</v>
+      </c>
+      <c r="K9" s="10">
+        <v>0.85050000000000003</v>
+      </c>
+      <c r="L9" s="10">
+        <v>0.91</v>
+      </c>
+      <c r="M9" s="1"/>
+    </row>
+    <row r="10" spans="1:14">
+      <c r="A10" s="3" t="s">
+        <v>20</v>
+      </c>
+      <c r="B10" s="3" t="s">
+        <v>13</v>
+      </c>
+      <c r="C10" s="3">
+        <v>1</v>
+      </c>
+      <c r="D10" s="3">
+        <v>0</v>
+      </c>
+      <c r="E10" s="3">
+        <v>0</v>
+      </c>
+      <c r="F10" s="3" t="s">
+        <v>25</v>
+      </c>
+      <c r="G10" s="10">
+        <v>0.88480000000000003</v>
+      </c>
+      <c r="H10" s="10">
+        <v>0.95630000000000004</v>
+      </c>
+      <c r="I10" s="10">
+        <v>0.95699999999999996</v>
+      </c>
+      <c r="J10" s="10">
+        <v>0.79169999999999996</v>
+      </c>
+      <c r="K10" s="10">
+        <v>0.85580000000000001</v>
+      </c>
+      <c r="L10" s="10">
+        <v>0.90359999999999996</v>
+      </c>
+      <c r="M10" s="1"/>
+    </row>
+    <row r="11" spans="1:14">
+      <c r="A11" s="3" t="s">
+        <v>28</v>
+      </c>
+      <c r="B11" s="3" t="s">
+        <v>10</v>
+      </c>
+      <c r="C11" s="3">
+        <v>1</v>
+      </c>
+      <c r="D11" s="3">
+        <v>0</v>
+      </c>
+      <c r="E11" s="3">
+        <v>1</v>
+      </c>
+      <c r="F11" s="3" t="s">
+        <v>25</v>
+      </c>
+      <c r="G11" s="10">
+        <v>0.92120000000000002</v>
+      </c>
+      <c r="H11" s="10">
+        <v>0.9698</v>
+      </c>
+      <c r="I11" s="10">
+        <v>0.95699999999999996</v>
+      </c>
+      <c r="J11" s="10">
+        <v>0.875</v>
+      </c>
+      <c r="K11" s="10">
+        <v>0.90820000000000001</v>
+      </c>
+      <c r="L11" s="10">
+        <v>0.93189999999999995</v>
+      </c>
+      <c r="M11" s="1"/>
+    </row>
+    <row r="12" spans="1:14">
+      <c r="A12" s="3" t="s">
+        <v>21</v>
+      </c>
+      <c r="B12" s="3" t="s">
+        <v>14</v>
+      </c>
+      <c r="C12" s="3">
+        <v>0</v>
+      </c>
+      <c r="D12" s="3">
+        <v>1</v>
+      </c>
+      <c r="E12" s="3">
+        <v>0</v>
+      </c>
+      <c r="F12" s="3" t="s">
+        <v>25</v>
+      </c>
+      <c r="G12" s="10">
+        <v>0.90910000000000002</v>
+      </c>
+      <c r="H12" s="10">
+        <v>0.96399999999999997</v>
+      </c>
+      <c r="I12" s="10">
+        <v>0.91400000000000003</v>
+      </c>
+      <c r="J12" s="10">
+        <v>0.90280000000000005</v>
+      </c>
+      <c r="K12" s="10">
+        <v>0.92390000000000005</v>
+      </c>
+      <c r="L12" s="10">
+        <v>0.91890000000000005</v>
+      </c>
+      <c r="M12" s="1"/>
+    </row>
+    <row r="13" spans="1:14">
+      <c r="A13" s="3" t="s">
+        <v>29</v>
+      </c>
+      <c r="B13" s="3" t="s">
+        <v>17</v>
+      </c>
+      <c r="C13" s="3">
+        <v>0</v>
+      </c>
+      <c r="D13" s="3">
+        <v>1</v>
+      </c>
+      <c r="E13" s="3">
+        <v>1</v>
+      </c>
+      <c r="F13" s="3" t="s">
+        <v>25</v>
+      </c>
+      <c r="G13" s="10">
+        <v>0.92730000000000001</v>
+      </c>
+      <c r="H13" s="10">
+        <v>0.97450000000000003</v>
+      </c>
+      <c r="I13" s="10">
+        <v>0.91400000000000003</v>
+      </c>
+      <c r="J13" s="10">
+        <v>0.94440000000000002</v>
+      </c>
+      <c r="K13" s="10">
+        <v>0.95509999999999995</v>
+      </c>
+      <c r="L13" s="10">
+        <v>0.93410000000000004</v>
+      </c>
+      <c r="M13" s="1"/>
+    </row>
+    <row r="14" spans="1:14">
+      <c r="A14" s="3" t="s">
+        <v>22</v>
+      </c>
+      <c r="B14" s="3" t="s">
+        <v>15</v>
+      </c>
+      <c r="C14" s="3">
+        <v>1</v>
+      </c>
+      <c r="D14" s="3">
+        <v>1</v>
+      </c>
+      <c r="E14" s="3">
+        <v>0</v>
+      </c>
+      <c r="F14" s="3" t="s">
+        <v>25</v>
+      </c>
+      <c r="G14" s="10">
+        <v>0.89090000000000003</v>
+      </c>
+      <c r="H14" s="10">
+        <v>0.97009999999999996</v>
+      </c>
+      <c r="I14" s="10">
+        <v>0.94620000000000004</v>
+      </c>
+      <c r="J14" s="10">
+        <v>0.81940000000000002</v>
+      </c>
+      <c r="K14" s="10">
+        <v>0.87129999999999996</v>
+      </c>
+      <c r="L14" s="10">
+        <v>0.90720000000000001</v>
+      </c>
+      <c r="M14" s="1"/>
+    </row>
+    <row r="15" spans="1:14">
+      <c r="A15" s="3" t="s">
+        <v>30</v>
+      </c>
+      <c r="B15" s="3" t="s">
+        <v>11</v>
+      </c>
+      <c r="C15" s="3">
+        <v>1</v>
+      </c>
+      <c r="D15" s="3">
+        <v>1</v>
+      </c>
+      <c r="E15" s="3">
+        <v>1</v>
+      </c>
+      <c r="F15" s="3" t="s">
+        <v>25</v>
+      </c>
+      <c r="G15" s="11">
+        <v>0.93940000000000001</v>
+      </c>
+      <c r="H15" s="11">
+        <v>0.97140000000000004</v>
+      </c>
+      <c r="I15" s="11">
+        <v>0.9355</v>
+      </c>
+      <c r="J15" s="11">
+        <v>0.94440000000000002</v>
+      </c>
+      <c r="K15" s="11">
+        <v>0.95599999999999996</v>
+      </c>
+      <c r="L15" s="11">
+        <v>0.94569999999999999</v>
+      </c>
+      <c r="M15" s="1"/>
+    </row>
+    <row r="16" spans="1:14">
+      <c r="A16" s="4" t="s">
+        <v>19</v>
+      </c>
+      <c r="B16" s="4" t="s">
+        <v>12</v>
+      </c>
+      <c r="C16" s="4">
+        <v>0</v>
+      </c>
+      <c r="D16" s="4">
+        <v>0</v>
+      </c>
+      <c r="E16" s="4">
+        <v>1</v>
+      </c>
+      <c r="F16" s="4" t="s">
+        <v>26</v>
+      </c>
+      <c r="G16" s="5">
+        <v>0.81869999999999998</v>
+      </c>
+      <c r="H16" s="5">
+        <v>0.95369999999999999</v>
+      </c>
+      <c r="I16" s="5">
+        <v>0.96250000000000002</v>
+      </c>
+      <c r="J16" s="5">
+        <v>0.67500000000000004</v>
+      </c>
+      <c r="K16" s="5">
+        <v>0.74760000000000004</v>
+      </c>
+      <c r="L16" s="5">
+        <v>0.84150000000000003</v>
+      </c>
+      <c r="M16" s="1"/>
+    </row>
+    <row r="17" spans="1:13">
+      <c r="A17" s="4" t="s">
+        <v>20</v>
+      </c>
+      <c r="B17" s="4" t="s">
+        <v>13</v>
+      </c>
+      <c r="C17" s="4">
+        <v>1</v>
+      </c>
+      <c r="D17" s="4">
+        <v>0</v>
+      </c>
+      <c r="E17" s="4">
+        <v>0</v>
+      </c>
+      <c r="F17" s="4" t="s">
+        <v>26</v>
+      </c>
+      <c r="G17" s="5">
+        <v>0.82499999999999996</v>
+      </c>
+      <c r="H17" s="5">
+        <v>0.91700000000000004</v>
+      </c>
+      <c r="I17" s="5">
+        <v>0.9375</v>
+      </c>
+      <c r="J17" s="5">
+        <v>0.71250000000000002</v>
+      </c>
+      <c r="K17" s="5">
+        <v>0.76529999999999998</v>
+      </c>
+      <c r="L17" s="5">
+        <v>0.8427</v>
+      </c>
+      <c r="M17" s="1"/>
+    </row>
+    <row r="18" spans="1:13">
+      <c r="A18" s="4" t="s">
+        <v>28</v>
+      </c>
+      <c r="B18" s="4" t="s">
+        <v>10</v>
+      </c>
+      <c r="C18" s="4">
+        <v>1</v>
+      </c>
+      <c r="D18" s="4">
+        <v>0</v>
+      </c>
+      <c r="E18" s="4">
+        <v>1</v>
+      </c>
+      <c r="F18" s="4" t="s">
+        <v>26</v>
+      </c>
+      <c r="G18" s="5">
+        <v>0.83130000000000004</v>
+      </c>
+      <c r="H18" s="5">
+        <v>0.91059999999999997</v>
+      </c>
+      <c r="I18" s="5">
+        <v>0.9</v>
+      </c>
+      <c r="J18" s="5">
+        <v>0.76249999999999996</v>
+      </c>
+      <c r="K18" s="5">
+        <v>0.79120000000000001</v>
+      </c>
+      <c r="L18" s="5">
+        <v>0.84209999999999996</v>
+      </c>
+      <c r="M18" s="1"/>
+    </row>
+    <row r="19" spans="1:13">
+      <c r="A19" s="4" t="s">
+        <v>21</v>
+      </c>
+      <c r="B19" s="4" t="s">
+        <v>14</v>
+      </c>
+      <c r="C19" s="4">
+        <v>0</v>
+      </c>
+      <c r="D19" s="4">
+        <v>1</v>
+      </c>
+      <c r="E19" s="4">
+        <v>0</v>
+      </c>
+      <c r="F19" s="4" t="s">
+        <v>26</v>
+      </c>
+      <c r="G19" s="5">
+        <v>0.83130000000000004</v>
+      </c>
+      <c r="H19" s="5">
+        <v>0.91910000000000003</v>
+      </c>
+      <c r="I19" s="5">
+        <v>0.82499999999999996</v>
+      </c>
+      <c r="J19" s="5">
+        <v>0.83750000000000002</v>
+      </c>
+      <c r="K19" s="5">
+        <v>0.83540000000000003</v>
+      </c>
+      <c r="L19" s="5">
+        <v>0.83020000000000005</v>
+      </c>
+      <c r="M19" s="1"/>
+    </row>
+    <row r="20" spans="1:13">
+      <c r="A20" s="4" t="s">
+        <v>29</v>
+      </c>
+      <c r="B20" s="4" t="s">
+        <v>17</v>
+      </c>
+      <c r="C20" s="4">
+        <v>0</v>
+      </c>
+      <c r="D20" s="4">
+        <v>1</v>
+      </c>
+      <c r="E20" s="4">
+        <v>1</v>
+      </c>
+      <c r="F20" s="4" t="s">
+        <v>26</v>
+      </c>
+      <c r="G20" s="5">
+        <v>0.82499999999999996</v>
+      </c>
+      <c r="H20" s="5">
+        <v>0.90669999999999995</v>
+      </c>
+      <c r="I20" s="5">
+        <v>0.78749999999999998</v>
+      </c>
+      <c r="J20" s="5">
+        <v>0.86250000000000004</v>
+      </c>
+      <c r="K20" s="5">
+        <v>0.85140000000000005</v>
+      </c>
+      <c r="L20" s="5">
+        <v>0.81820000000000004</v>
+      </c>
+      <c r="M20" s="1"/>
+    </row>
+    <row r="21" spans="1:13">
+      <c r="A21" s="4" t="s">
+        <v>22</v>
+      </c>
+      <c r="B21" s="4" t="s">
+        <v>15</v>
+      </c>
+      <c r="C21" s="4">
+        <v>1</v>
+      </c>
+      <c r="D21" s="4">
+        <v>1</v>
+      </c>
+      <c r="E21" s="4">
+        <v>0</v>
+      </c>
+      <c r="F21" s="4" t="s">
+        <v>26</v>
+      </c>
+      <c r="G21" s="5">
+        <v>0.85619999999999996</v>
+      </c>
+      <c r="H21" s="5">
+        <v>0.91869999999999996</v>
+      </c>
+      <c r="I21" s="5">
+        <v>0.86250000000000004</v>
+      </c>
+      <c r="J21" s="5">
+        <v>0.85</v>
+      </c>
+      <c r="K21" s="5">
+        <v>0.85189999999999999</v>
+      </c>
+      <c r="L21" s="5">
+        <v>0.85709999999999997</v>
+      </c>
+      <c r="M21" s="1"/>
+    </row>
+    <row r="22" spans="1:13">
+      <c r="A22" s="4" t="s">
+        <v>30</v>
+      </c>
+      <c r="B22" s="4" t="s">
+        <v>11</v>
+      </c>
+      <c r="C22" s="4">
+        <v>1</v>
+      </c>
+      <c r="D22" s="4">
+        <v>1</v>
+      </c>
+      <c r="E22" s="4">
+        <v>1</v>
+      </c>
+      <c r="F22" s="4" t="s">
+        <v>26</v>
+      </c>
+      <c r="G22" s="5">
+        <v>0.90620000000000001</v>
+      </c>
+      <c r="H22" s="5">
+        <v>0.96050000000000002</v>
+      </c>
+      <c r="I22" s="5">
+        <v>0.83750000000000002</v>
+      </c>
+      <c r="J22" s="5">
+        <v>0.97499999999999998</v>
+      </c>
+      <c r="K22" s="5">
+        <v>0.97099999999999997</v>
+      </c>
+      <c r="L22" s="5">
+        <v>0.89929999999999999</v>
+      </c>
+      <c r="M22" s="1"/>
+    </row>
+    <row r="23" spans="1:13">
+      <c r="A23" s="6" t="s">
+        <v>19</v>
+      </c>
+      <c r="B23" s="6" t="s">
+        <v>12</v>
+      </c>
+      <c r="C23" s="6">
+        <v>0</v>
+      </c>
+      <c r="D23" s="6">
+        <v>0</v>
+      </c>
+      <c r="E23" s="6">
+        <v>1</v>
+      </c>
+      <c r="F23" s="6" t="s">
+        <v>27</v>
+      </c>
+      <c r="G23" s="7">
+        <v>0.67210000000000003</v>
+      </c>
+      <c r="H23" s="7"/>
+      <c r="I23" s="7"/>
+      <c r="J23" s="7">
+        <v>0.67210000000000003</v>
+      </c>
+      <c r="K23" s="7"/>
+      <c r="L23" s="7"/>
+      <c r="M23" s="1"/>
+    </row>
+    <row r="24" spans="1:13">
+      <c r="A24" s="6" t="s">
+        <v>20</v>
+      </c>
+      <c r="B24" s="6" t="s">
+        <v>13</v>
+      </c>
+      <c r="C24" s="6">
+        <v>1</v>
+      </c>
+      <c r="D24" s="6">
+        <v>0</v>
+      </c>
+      <c r="E24" s="6">
+        <v>0</v>
+      </c>
+      <c r="F24" s="6" t="s">
+        <v>27</v>
+      </c>
+      <c r="G24" s="7">
+        <v>0.73770000000000002</v>
+      </c>
+      <c r="H24" s="7"/>
+      <c r="I24" s="7"/>
+      <c r="J24" s="7">
+        <v>0.73770000000000002</v>
+      </c>
+      <c r="K24" s="7"/>
+      <c r="L24" s="7"/>
+      <c r="M24" s="1"/>
+    </row>
+    <row r="25" spans="1:13">
+      <c r="A25" s="6" t="s">
+        <v>28</v>
+      </c>
+      <c r="B25" s="6" t="s">
+        <v>10</v>
+      </c>
+      <c r="C25" s="6">
+        <v>1</v>
+      </c>
+      <c r="D25" s="6">
+        <v>0</v>
+      </c>
+      <c r="E25" s="6">
+        <v>1</v>
+      </c>
+      <c r="F25" s="6" t="s">
+        <v>27</v>
+      </c>
+      <c r="G25" s="7">
+        <v>0.78690000000000004</v>
+      </c>
+      <c r="H25" s="7"/>
+      <c r="I25" s="7"/>
+      <c r="J25" s="7">
+        <v>0.78690000000000004</v>
+      </c>
+      <c r="K25" s="7"/>
+      <c r="L25" s="7"/>
+      <c r="M25" s="1"/>
+    </row>
+    <row r="26" spans="1:13">
+      <c r="A26" s="6" t="s">
+        <v>21</v>
+      </c>
+      <c r="B26" s="6" t="s">
+        <v>14</v>
+      </c>
+      <c r="C26" s="6">
+        <v>0</v>
+      </c>
+      <c r="D26" s="6">
+        <v>1</v>
+      </c>
+      <c r="E26" s="6">
+        <v>0</v>
+      </c>
+      <c r="F26" s="6" t="s">
+        <v>27</v>
+      </c>
+      <c r="G26" s="7">
+        <v>0.90159999999999996</v>
+      </c>
+      <c r="H26" s="7"/>
+      <c r="I26" s="7"/>
+      <c r="J26" s="7">
+        <v>0.90159999999999996</v>
+      </c>
+      <c r="K26" s="7"/>
+      <c r="L26" s="7"/>
+      <c r="M26" s="1"/>
+    </row>
+    <row r="27" spans="1:13">
+      <c r="A27" s="6" t="s">
+        <v>29</v>
+      </c>
+      <c r="B27" s="6" t="s">
+        <v>17</v>
+      </c>
+      <c r="C27" s="6">
+        <v>0</v>
+      </c>
+      <c r="D27" s="6">
+        <v>1</v>
+      </c>
+      <c r="E27" s="6">
+        <v>1</v>
+      </c>
+      <c r="F27" s="6" t="s">
+        <v>27</v>
+      </c>
+      <c r="G27" s="7">
+        <v>0.91800000000000004</v>
+      </c>
+      <c r="H27" s="7"/>
+      <c r="I27" s="7"/>
+      <c r="J27" s="7">
+        <v>0.91800000000000004</v>
+      </c>
+      <c r="K27" s="7"/>
+      <c r="L27" s="7"/>
+      <c r="M27" s="1"/>
+    </row>
+    <row r="28" spans="1:13">
+      <c r="A28" s="6" t="s">
+        <v>22</v>
+      </c>
+      <c r="B28" s="6" t="s">
+        <v>15</v>
+      </c>
+      <c r="C28" s="6">
+        <v>1</v>
+      </c>
+      <c r="D28" s="6">
+        <v>1</v>
+      </c>
+      <c r="E28" s="6">
+        <v>0</v>
+      </c>
+      <c r="F28" s="6" t="s">
+        <v>27</v>
+      </c>
+      <c r="G28" s="7">
+        <v>0.90159999999999996</v>
+      </c>
+      <c r="H28" s="7"/>
+      <c r="I28" s="7"/>
+      <c r="J28" s="7">
+        <v>0.90159999999999996</v>
+      </c>
+      <c r="K28" s="7"/>
+      <c r="L28" s="7"/>
+      <c r="M28" s="1"/>
+    </row>
+    <row r="29" spans="1:13">
+      <c r="A29" s="6" t="s">
+        <v>30</v>
+      </c>
+      <c r="B29" s="6" t="s">
+        <v>11</v>
+      </c>
+      <c r="C29" s="6">
+        <v>1</v>
+      </c>
+      <c r="D29" s="6">
+        <v>1</v>
+      </c>
+      <c r="E29" s="6">
+        <v>1</v>
+      </c>
+      <c r="F29" s="6" t="s">
+        <v>27</v>
+      </c>
+      <c r="G29" s="7">
+        <v>0.93440000000000001</v>
+      </c>
+      <c r="H29" s="7"/>
+      <c r="I29" s="7"/>
+      <c r="J29" s="7">
+        <v>0.93440000000000001</v>
+      </c>
+      <c r="K29" s="7"/>
+      <c r="L29" s="7"/>
+      <c r="M29" s="1"/>
+    </row>
+    <row r="34" spans="7:12">
+      <c r="G34" s="8"/>
+      <c r="H34" s="8"/>
+      <c r="I34" s="8"/>
+      <c r="J34" s="8"/>
+      <c r="K34" s="8"/>
+      <c r="L34" s="8"/>
+    </row>
+    <row r="35" spans="7:12">
+      <c r="G35" s="8"/>
+      <c r="H35" s="8"/>
+      <c r="I35" s="8"/>
+      <c r="J35" s="8"/>
+      <c r="K35" s="8"/>
+      <c r="L35" s="8"/>
+    </row>
+    <row r="36" spans="7:12">
+      <c r="G36" s="8"/>
+      <c r="H36" s="8"/>
+      <c r="I36" s="8"/>
+      <c r="J36" s="8"/>
+      <c r="K36" s="8"/>
+      <c r="L36" s="8"/>
+    </row>
+    <row r="37" spans="7:12">
+      <c r="G37" s="8"/>
+      <c r="H37" s="8"/>
+      <c r="I37" s="8"/>
+      <c r="J37" s="8"/>
+      <c r="K37" s="8"/>
+      <c r="L37" s="8"/>
+    </row>
+    <row r="38" spans="7:12">
+      <c r="G38" s="8"/>
+      <c r="H38" s="8"/>
+      <c r="I38" s="8"/>
+      <c r="J38" s="8"/>
+      <c r="K38" s="8"/>
+      <c r="L38" s="8"/>
+    </row>
+    <row r="39" spans="7:12">
+      <c r="G39" s="8"/>
+      <c r="H39" s="8"/>
+      <c r="I39" s="8"/>
+      <c r="J39" s="8"/>
+      <c r="K39" s="8"/>
+      <c r="L39" s="8"/>
+    </row>
+    <row r="40" spans="7:12">
+      <c r="G40" s="8"/>
+      <c r="H40" s="8"/>
+      <c r="I40" s="8"/>
+      <c r="J40" s="8"/>
+      <c r="K40" s="8"/>
+      <c r="L40" s="8"/>
+    </row>
+    <row r="41" spans="7:12">
+      <c r="G41" s="8"/>
+      <c r="H41" s="8"/>
+      <c r="I41" s="8"/>
+      <c r="J41" s="8"/>
+      <c r="K41" s="8"/>
+      <c r="L41" s="8"/>
+    </row>
+    <row r="42" spans="7:12">
+      <c r="G42" s="8"/>
+      <c r="H42" s="8"/>
+      <c r="I42" s="8"/>
+      <c r="J42" s="8"/>
+      <c r="K42" s="8"/>
+      <c r="L42" s="8"/>
+    </row>
+    <row r="43" spans="7:12">
+      <c r="G43" s="8"/>
+      <c r="H43" s="8"/>
+      <c r="I43" s="8"/>
+      <c r="J43" s="8"/>
+      <c r="K43" s="8"/>
+      <c r="L43" s="8"/>
+    </row>
+    <row r="44" spans="7:12">
+      <c r="G44" s="8"/>
+      <c r="H44" s="8"/>
+      <c r="I44" s="8"/>
+      <c r="J44" s="8"/>
+      <c r="K44" s="8"/>
+      <c r="L44" s="8"/>
+    </row>
+    <row r="45" spans="7:12">
+      <c r="G45" s="8"/>
+      <c r="H45" s="8"/>
+      <c r="I45" s="8"/>
+      <c r="J45" s="8"/>
+      <c r="K45" s="8"/>
+      <c r="L45" s="8"/>
+    </row>
+  </sheetData>
   <phoneticPr fontId="1" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup paperSize="9" orientation="portrait" horizontalDpi="0" verticalDpi="0"/>
 </worksheet>
 </file>
</xml_diff>